<commit_message>
Benchmarks have been updated. Outputs have been updated.
</commit_message>
<xml_diff>
--- a/outputs/benchmark_report.xlsx
+++ b/outputs/benchmark_report.xlsx
@@ -482,22 +482,22 @@
         <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>21.91</v>
+        <v>22.94</v>
       </c>
       <c r="C2" t="n">
-        <v>30.99</v>
+        <v>32.1</v>
       </c>
       <c r="D2" t="n">
-        <v>26.82</v>
+        <v>29.98</v>
       </c>
       <c r="E2" t="n">
-        <v>42.05</v>
+        <v>44.12</v>
       </c>
       <c r="F2" t="n">
-        <v>453.78</v>
+        <v>433.53</v>
       </c>
       <c r="G2" t="n">
-        <v>320.85</v>
+        <v>309.91</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -506,7 +506,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>-9.08</v>
+        <v>-9.16</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -519,22 +519,22 @@
         <v>50</v>
       </c>
       <c r="B3" t="n">
-        <v>109.18</v>
+        <v>113.9</v>
       </c>
       <c r="C3" t="n">
-        <v>146.8</v>
+        <v>155.37</v>
       </c>
       <c r="D3" t="n">
-        <v>118.75</v>
+        <v>126.84</v>
       </c>
       <c r="E3" t="n">
-        <v>184.31</v>
+        <v>200.99</v>
       </c>
       <c r="F3" t="n">
-        <v>457.5</v>
+        <v>438.6</v>
       </c>
       <c r="G3" t="n">
-        <v>340.25</v>
+        <v>321.91</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>-37.62</v>
+        <v>-41.47</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -556,22 +556,22 @@
         <v>100</v>
       </c>
       <c r="B4" t="n">
-        <v>217.6</v>
+        <v>231.04</v>
       </c>
       <c r="C4" t="n">
-        <v>289.25</v>
+        <v>306.83</v>
       </c>
       <c r="D4" t="n">
-        <v>226.19</v>
+        <v>244.4</v>
       </c>
       <c r="E4" t="n">
-        <v>362.91</v>
+        <v>390.75</v>
       </c>
       <c r="F4" t="n">
-        <v>459.3</v>
+        <v>432.92</v>
       </c>
       <c r="G4" t="n">
-        <v>345.49</v>
+        <v>326.14</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -580,7 +580,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>-71.65000000000001</v>
+        <v>-75.79000000000001</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -593,31 +593,31 @@
         <v>200</v>
       </c>
       <c r="B5" t="n">
-        <v>437.07</v>
+        <v>465.43</v>
       </c>
       <c r="C5" t="n">
-        <v>571.62</v>
+        <v>615.08</v>
       </c>
       <c r="D5" t="n">
-        <v>453.43</v>
+        <v>482.05</v>
       </c>
       <c r="E5" t="n">
-        <v>640.22</v>
+        <v>780.92</v>
       </c>
       <c r="F5" t="n">
-        <v>457.39</v>
+        <v>429.92</v>
       </c>
       <c r="G5" t="n">
-        <v>349.68</v>
+        <v>325.18</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="J5" t="n">
-        <v>-134.55</v>
+        <v>-149.65</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -701,22 +701,22 @@
         <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>58.16</v>
+        <v>51</v>
       </c>
       <c r="C2" t="n">
-        <v>28.24</v>
+        <v>29.62</v>
       </c>
       <c r="D2" t="n">
-        <v>76.23999999999999</v>
+        <v>65.33</v>
       </c>
       <c r="E2" t="n">
-        <v>36.06</v>
+        <v>39.01</v>
       </c>
       <c r="F2" t="n">
-        <v>171.25</v>
+        <v>195.24</v>
       </c>
       <c r="G2" t="n">
-        <v>352.1</v>
+        <v>335.72</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -725,7 +725,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>29.92</v>
+        <v>21.38</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -738,22 +738,22 @@
         <v>50</v>
       </c>
       <c r="B3" t="n">
-        <v>287.53</v>
+        <v>251.58</v>
       </c>
       <c r="C3" t="n">
-        <v>140.13</v>
+        <v>146.91</v>
       </c>
       <c r="D3" t="n">
-        <v>334.39</v>
+        <v>287.44</v>
       </c>
       <c r="E3" t="n">
-        <v>198.79</v>
+        <v>211.42</v>
       </c>
       <c r="F3" t="n">
-        <v>173.69</v>
+        <v>198.52</v>
       </c>
       <c r="G3" t="n">
-        <v>356.4</v>
+        <v>339.96</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -762,7 +762,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>147.4</v>
+        <v>104.67</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -775,31 +775,31 @@
         <v>100</v>
       </c>
       <c r="B4" t="n">
-        <v>576.27</v>
+        <v>497.19</v>
       </c>
       <c r="C4" t="n">
-        <v>284.68</v>
+        <v>292.18</v>
       </c>
       <c r="D4" t="n">
-        <v>640.55</v>
+        <v>533.45</v>
       </c>
       <c r="E4" t="n">
-        <v>404.92</v>
+        <v>417</v>
       </c>
       <c r="F4" t="n">
-        <v>173.36</v>
+        <v>200.93</v>
       </c>
       <c r="G4" t="n">
-        <v>351.03</v>
+        <v>342.02</v>
       </c>
       <c r="H4" t="n">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>291.59</v>
+        <v>205.01</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -812,31 +812,31 @@
         <v>200</v>
       </c>
       <c r="B5" t="n">
-        <v>1154.35</v>
+        <v>997.8</v>
       </c>
       <c r="C5" t="n">
-        <v>566.23</v>
+        <v>608.8099999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>1237.71</v>
+        <v>1049.18</v>
       </c>
       <c r="E5" t="n">
-        <v>765.36</v>
+        <v>838.63</v>
       </c>
       <c r="F5" t="n">
-        <v>173</v>
+        <v>200.17</v>
       </c>
       <c r="G5" t="n">
-        <v>352.96</v>
+        <v>328.43</v>
       </c>
       <c r="H5" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I5" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J5" t="n">
-        <v>588.12</v>
+        <v>388.99</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -920,22 +920,22 @@
         <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>168.29</v>
+        <v>167.53</v>
       </c>
       <c r="C2" t="n">
-        <v>166.28</v>
+        <v>172.54</v>
       </c>
       <c r="D2" t="n">
-        <v>193.25</v>
+        <v>192.38</v>
       </c>
       <c r="E2" t="n">
-        <v>190.43</v>
+        <v>197.28</v>
       </c>
       <c r="F2" t="n">
-        <v>59.34</v>
+        <v>59.61</v>
       </c>
       <c r="G2" t="n">
-        <v>60.05</v>
+        <v>57.88</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -944,11 +944,11 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2.01</v>
+        <v>-5.01</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -957,22 +957,22 @@
         <v>50</v>
       </c>
       <c r="B3" t="n">
-        <v>845.41</v>
+        <v>841.3099999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>831.2</v>
+        <v>876.16</v>
       </c>
       <c r="D3" t="n">
-        <v>876.54</v>
+        <v>871.78</v>
       </c>
       <c r="E3" t="n">
-        <v>859.54</v>
+        <v>915.3200000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>59.05</v>
+        <v>59.34</v>
       </c>
       <c r="G3" t="n">
-        <v>60.06</v>
+        <v>56.97</v>
       </c>
       <c r="H3" t="n">
         <v>100</v>
@@ -981,11 +981,11 @@
         <v>100</v>
       </c>
       <c r="J3" t="n">
-        <v>14.21</v>
+        <v>-34.85</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -994,22 +994,22 @@
         <v>100</v>
       </c>
       <c r="B4" t="n">
-        <v>1687.15</v>
+        <v>1739.72</v>
       </c>
       <c r="C4" t="n">
-        <v>1658.58</v>
+        <v>1737.51</v>
       </c>
       <c r="D4" t="n">
-        <v>1727.91</v>
+        <v>1839.3</v>
       </c>
       <c r="E4" t="n">
-        <v>1679.94</v>
+        <v>1790.45</v>
       </c>
       <c r="F4" t="n">
-        <v>59.11</v>
+        <v>57.32</v>
       </c>
       <c r="G4" t="n">
-        <v>60.12</v>
+        <v>57.39</v>
       </c>
       <c r="H4" t="n">
         <v>100</v>
@@ -1018,7 +1018,7 @@
         <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>28.57</v>
+        <v>2.21</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1031,22 +1031,22 @@
         <v>200</v>
       </c>
       <c r="B5" t="n">
-        <v>3359.53</v>
+        <v>3408.5</v>
       </c>
       <c r="C5" t="n">
-        <v>3309.1</v>
+        <v>3494</v>
       </c>
       <c r="D5" t="n">
-        <v>3433.74</v>
+        <v>3472.08</v>
       </c>
       <c r="E5" t="n">
-        <v>3348.78</v>
+        <v>3583.26</v>
       </c>
       <c r="F5" t="n">
-        <v>59.2</v>
+        <v>58.34</v>
       </c>
       <c r="G5" t="n">
-        <v>60.11</v>
+        <v>56.91</v>
       </c>
       <c r="H5" t="n">
         <v>100</v>
@@ -1055,11 +1055,11 @@
         <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>50.43</v>
+        <v>-85.5</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1139,22 +1139,22 @@
         <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>18.36</v>
+        <v>16.44</v>
       </c>
       <c r="C2" t="n">
-        <v>16.16</v>
+        <v>17.6</v>
       </c>
       <c r="D2" t="n">
-        <v>24.17</v>
+        <v>21.19</v>
       </c>
       <c r="E2" t="n">
-        <v>21.72</v>
+        <v>24.6</v>
       </c>
       <c r="F2" t="n">
-        <v>541.0599999999999</v>
+        <v>604.24</v>
       </c>
       <c r="G2" t="n">
-        <v>613.12</v>
+        <v>563.3099999999999</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1163,11 +1163,11 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2.2</v>
+        <v>-1.16</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1176,22 +1176,22 @@
         <v>50</v>
       </c>
       <c r="B3" t="n">
-        <v>90.76000000000001</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>82.40000000000001</v>
+        <v>85.06</v>
       </c>
       <c r="D3" t="n">
-        <v>102.74</v>
+        <v>89.65000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>92.98</v>
+        <v>99.63</v>
       </c>
       <c r="F3" t="n">
-        <v>550.23</v>
+        <v>618.52</v>
       </c>
       <c r="G3" t="n">
-        <v>605.65</v>
+        <v>586.86</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1200,11 +1200,11 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>8.359999999999999</v>
+        <v>-4.32</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1213,22 +1213,22 @@
         <v>100</v>
       </c>
       <c r="B4" t="n">
-        <v>180.82</v>
+        <v>157.18</v>
       </c>
       <c r="C4" t="n">
-        <v>162.52</v>
+        <v>163.93</v>
       </c>
       <c r="D4" t="n">
-        <v>204.25</v>
+        <v>171.29</v>
       </c>
       <c r="E4" t="n">
-        <v>182.67</v>
+        <v>188.25</v>
       </c>
       <c r="F4" t="n">
-        <v>552.97</v>
+        <v>635.73</v>
       </c>
       <c r="G4" t="n">
-        <v>614.72</v>
+        <v>609.35</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -1237,11 +1237,11 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>18.3</v>
+        <v>-6.75</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1250,22 +1250,22 @@
         <v>200</v>
       </c>
       <c r="B5" t="n">
-        <v>358.69</v>
+        <v>309.64</v>
       </c>
       <c r="C5" t="n">
-        <v>317.31</v>
+        <v>321.57</v>
       </c>
       <c r="D5" t="n">
-        <v>397.3</v>
+        <v>329.57</v>
       </c>
       <c r="E5" t="n">
-        <v>344.43</v>
+        <v>357.65</v>
       </c>
       <c r="F5" t="n">
-        <v>557.73</v>
+        <v>645.53</v>
       </c>
       <c r="G5" t="n">
-        <v>629.79</v>
+        <v>621.53</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -1274,11 +1274,11 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>41.38</v>
+        <v>-11.93</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1378,29 +1378,29 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>21.9072</v>
+        <v>22.939</v>
       </c>
       <c r="D2" t="n">
-        <v>30.9902</v>
+        <v>32.0973</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1558</v>
+        <v>0.1717</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2695</v>
+        <v>0.8512</v>
       </c>
       <c r="G2" t="n">
-        <v>0.387</v>
+        <v>0.4266</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6694</v>
+        <v>2.1144</v>
       </c>
       <c r="I2" t="n">
-        <v>-50.5456</v>
+        <v>-18.2683</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>&lt; 0.001</t>
+          <t>0.002</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1409,7 +1409,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>41.27</v>
+        <v>14.92</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -1432,29 +1432,29 @@
         <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>109.1814</v>
+        <v>113.9049</v>
       </c>
       <c r="D3" t="n">
-        <v>146.8042</v>
+        <v>155.3709</v>
       </c>
       <c r="E3" t="n">
-        <v>1.2561</v>
+        <v>2.121</v>
       </c>
       <c r="F3" t="n">
-        <v>1.1914</v>
+        <v>7.0283</v>
       </c>
       <c r="G3" t="n">
-        <v>3.1203</v>
+        <v>5.2689</v>
       </c>
       <c r="H3" t="n">
-        <v>2.9597</v>
+        <v>17.4593</v>
       </c>
       <c r="I3" t="n">
-        <v>-37.6399</v>
+        <v>-9.783099999999999</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>&lt; 0.001</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>30.73</v>
+        <v>7.99</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -1486,29 +1486,29 @@
         <v>100</v>
       </c>
       <c r="C4" t="n">
-        <v>217.5992</v>
+        <v>231.0414</v>
       </c>
       <c r="D4" t="n">
-        <v>289.2519</v>
+        <v>306.829</v>
       </c>
       <c r="E4" t="n">
-        <v>1.7697</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="F4" t="n">
-        <v>2.2514</v>
+        <v>14.1667</v>
       </c>
       <c r="G4" t="n">
-        <v>4.3961</v>
+        <v>20.0594</v>
       </c>
       <c r="H4" t="n">
-        <v>5.5929</v>
+        <v>35.192</v>
       </c>
       <c r="I4" t="n">
-        <v>-43.3379</v>
+        <v>-8.0501</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>&lt; 0.001</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>35.39</v>
+        <v>6.57</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -1540,25 +1540,25 @@
         <v>200</v>
       </c>
       <c r="C5" t="n">
-        <v>437.0723</v>
+        <v>465.434</v>
       </c>
       <c r="D5" t="n">
-        <v>571.6188</v>
+        <v>615.0842</v>
       </c>
       <c r="E5" t="n">
-        <v>1.045</v>
+        <v>18.295</v>
       </c>
       <c r="F5" t="n">
-        <v>4.4944</v>
+        <v>20.3224</v>
       </c>
       <c r="G5" t="n">
-        <v>2.5959</v>
+        <v>45.4473</v>
       </c>
       <c r="H5" t="n">
-        <v>11.1648</v>
+        <v>50.4837</v>
       </c>
       <c r="I5" t="n">
-        <v>-50.5042</v>
+        <v>-9.479200000000001</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>41.24</v>
+        <v>7.74</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1594,25 +1594,25 @@
         <v>10</v>
       </c>
       <c r="C6" t="n">
-        <v>58.16</v>
+        <v>51.0005</v>
       </c>
       <c r="D6" t="n">
-        <v>28.2364</v>
+        <v>29.6151</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1994</v>
+        <v>0.3285</v>
       </c>
       <c r="F6" t="n">
-        <v>0.302</v>
+        <v>0.4494</v>
       </c>
       <c r="G6" t="n">
-        <v>0.4954</v>
+        <v>0.8161</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7503</v>
+        <v>1.1164</v>
       </c>
       <c r="I6" t="n">
-        <v>143.2042</v>
+        <v>66.53870000000001</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>116.93</v>
+        <v>54.33</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1648,25 +1648,25 @@
         <v>50</v>
       </c>
       <c r="C7" t="n">
-        <v>287.5274</v>
+        <v>251.5815</v>
       </c>
       <c r="D7" t="n">
-        <v>140.1308</v>
+        <v>146.9127</v>
       </c>
       <c r="E7" t="n">
-        <v>1.6692</v>
+        <v>2.3042</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5603</v>
+        <v>0.8781</v>
       </c>
       <c r="G7" t="n">
-        <v>4.1465</v>
+        <v>5.724</v>
       </c>
       <c r="H7" t="n">
-        <v>1.3919</v>
+        <v>2.1813</v>
       </c>
       <c r="I7" t="n">
-        <v>144.9974</v>
+        <v>73.5206</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>118.39</v>
+        <v>60.03</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1702,25 +1702,25 @@
         <v>100</v>
       </c>
       <c r="C8" t="n">
-        <v>576.2745</v>
+        <v>497.1928</v>
       </c>
       <c r="D8" t="n">
-        <v>284.6817</v>
+        <v>292.1759</v>
       </c>
       <c r="E8" t="n">
-        <v>3.2143</v>
+        <v>1.3951</v>
       </c>
       <c r="F8" t="n">
-        <v>1.5165</v>
+        <v>1.1662</v>
       </c>
       <c r="G8" t="n">
-        <v>7.9849</v>
+        <v>3.4657</v>
       </c>
       <c r="H8" t="n">
-        <v>3.7671</v>
+        <v>2.897</v>
       </c>
       <c r="I8" t="n">
-        <v>142.1042</v>
+        <v>195.2874</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>116.03</v>
+        <v>159.45</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1756,25 +1756,25 @@
         <v>200</v>
       </c>
       <c r="C9" t="n">
-        <v>1154.3518</v>
+        <v>997.8037</v>
       </c>
       <c r="D9" t="n">
-        <v>566.2318</v>
+        <v>608.8069</v>
       </c>
       <c r="E9" t="n">
-        <v>6.9734</v>
+        <v>4.7438</v>
       </c>
       <c r="F9" t="n">
-        <v>4.4712</v>
+        <v>17.771</v>
       </c>
       <c r="G9" t="n">
-        <v>17.3228</v>
+        <v>11.7843</v>
       </c>
       <c r="H9" t="n">
-        <v>11.1072</v>
+        <v>44.1456</v>
       </c>
       <c r="I9" t="n">
-        <v>122.971</v>
+        <v>36.6309</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>100.41</v>
+        <v>29.91</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1810,29 +1810,29 @@
         <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>168.2898</v>
+        <v>167.5279</v>
       </c>
       <c r="D10" t="n">
-        <v>166.2843</v>
+        <v>172.5385</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1401</v>
+        <v>0.1051</v>
       </c>
       <c r="F10" t="n">
-        <v>0.3454</v>
+        <v>0.3814</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3481</v>
+        <v>0.2612</v>
       </c>
       <c r="H10" t="n">
-        <v>0.8581</v>
+        <v>0.9474</v>
       </c>
       <c r="I10" t="n">
-        <v>9.3178</v>
+        <v>-21.9365</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>7.61</v>
+        <v>17.91</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1864,29 +1864,29 @@
         <v>50</v>
       </c>
       <c r="C11" t="n">
-        <v>845.4108</v>
+        <v>841.3066</v>
       </c>
       <c r="D11" t="n">
-        <v>831.205</v>
+        <v>876.1563</v>
       </c>
       <c r="E11" t="n">
-        <v>3.6321</v>
+        <v>6.7395</v>
       </c>
       <c r="F11" t="n">
-        <v>3.5253</v>
+        <v>4.3701</v>
       </c>
       <c r="G11" t="n">
-        <v>9.0227</v>
+        <v>16.7418</v>
       </c>
       <c r="H11" t="n">
-        <v>8.757300000000001</v>
+        <v>10.856</v>
       </c>
       <c r="I11" t="n">
-        <v>4.8611</v>
+        <v>-7.5148</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>3.97</v>
+        <v>6.14</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -1918,47 +1918,47 @@
         <v>100</v>
       </c>
       <c r="C12" t="n">
-        <v>1687.1515</v>
+        <v>1739.7198</v>
       </c>
       <c r="D12" t="n">
-        <v>1658.5813</v>
+        <v>1737.5137</v>
       </c>
       <c r="E12" t="n">
-        <v>6.7131</v>
+        <v>27.6628</v>
       </c>
       <c r="F12" t="n">
-        <v>3.1467</v>
+        <v>18.8152</v>
       </c>
       <c r="G12" t="n">
-        <v>16.6762</v>
+        <v>68.7182</v>
       </c>
       <c r="H12" t="n">
-        <v>7.8169</v>
+        <v>46.7395</v>
       </c>
       <c r="I12" t="n">
-        <v>6.6745</v>
+        <v>0.1142</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.915</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>5.45</v>
+        <v>0.09</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Large</t>
+          <t>Negligible</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>No Significant Difference</t>
         </is>
       </c>
     </row>
@@ -1972,29 +1972,29 @@
         <v>200</v>
       </c>
       <c r="C13" t="n">
-        <v>3359.5275</v>
+        <v>3408.5001</v>
       </c>
       <c r="D13" t="n">
-        <v>3309.1049</v>
+        <v>3494.0021</v>
       </c>
       <c r="E13" t="n">
-        <v>3.692</v>
+        <v>1.6635</v>
       </c>
       <c r="F13" t="n">
-        <v>7.4832</v>
+        <v>4.3611</v>
       </c>
       <c r="G13" t="n">
-        <v>9.1715</v>
+        <v>4.1324</v>
       </c>
       <c r="H13" t="n">
-        <v>18.5892</v>
+        <v>10.8336</v>
       </c>
       <c r="I13" t="n">
-        <v>10.4663</v>
+        <v>-31.7279</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>&lt; 0.001</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>8.550000000000001</v>
+        <v>25.91</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -2026,29 +2026,29 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>18.362</v>
+        <v>16.4387</v>
       </c>
       <c r="D14" t="n">
-        <v>16.1579</v>
+        <v>17.598</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1997</v>
+        <v>0.0416</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2918</v>
+        <v>0.3408</v>
       </c>
       <c r="G14" t="n">
-        <v>0.496</v>
+        <v>0.1035</v>
       </c>
       <c r="H14" t="n">
-        <v>0.7248</v>
+        <v>0.8465</v>
       </c>
       <c r="I14" t="n">
-        <v>10.7971</v>
+        <v>-5.8489</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>&lt; 0.001</t>
+          <t>0.026</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>8.82</v>
+        <v>4.78</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -2080,29 +2080,29 @@
         <v>50</v>
       </c>
       <c r="C15" t="n">
-        <v>90.7616</v>
+        <v>80.74379999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>82.3991</v>
+        <v>85.06310000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3142</v>
+        <v>0.9185</v>
       </c>
       <c r="F15" t="n">
-        <v>0.273</v>
+        <v>1.4661</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7806</v>
+        <v>2.2817</v>
       </c>
       <c r="H15" t="n">
-        <v>0.6782</v>
+        <v>3.6419</v>
       </c>
       <c r="I15" t="n">
-        <v>34.7965</v>
+        <v>-4.3243</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>&lt; 0.001</t>
+          <t>0.018</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>28.41</v>
+        <v>3.53</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -2134,29 +2134,29 @@
         <v>100</v>
       </c>
       <c r="C16" t="n">
-        <v>180.8162</v>
+        <v>157.1795</v>
       </c>
       <c r="D16" t="n">
-        <v>162.5197</v>
+        <v>163.9348</v>
       </c>
       <c r="E16" t="n">
-        <v>5.4407</v>
+        <v>0.6975</v>
       </c>
       <c r="F16" t="n">
-        <v>2.5708</v>
+        <v>0.7933</v>
       </c>
       <c r="G16" t="n">
-        <v>13.5155</v>
+        <v>1.7327</v>
       </c>
       <c r="H16" t="n">
-        <v>6.3862</v>
+        <v>1.9706</v>
       </c>
       <c r="I16" t="n">
-        <v>5.2664</v>
+        <v>-11.0766</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0.015</t>
+          <t>&lt; 0.001</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>4.3</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>
@@ -2188,29 +2188,29 @@
         <v>200</v>
       </c>
       <c r="C17" t="n">
-        <v>358.6946</v>
+        <v>309.6399</v>
       </c>
       <c r="D17" t="n">
-        <v>317.3085</v>
+        <v>321.5698</v>
       </c>
       <c r="E17" t="n">
-        <v>13.3023</v>
+        <v>1.7094</v>
       </c>
       <c r="F17" t="n">
-        <v>1.0767</v>
+        <v>4.6972</v>
       </c>
       <c r="G17" t="n">
-        <v>33.0447</v>
+        <v>4.2463</v>
       </c>
       <c r="H17" t="n">
-        <v>2.6747</v>
+        <v>11.6685</v>
       </c>
       <c r="I17" t="n">
-        <v>5.3712</v>
+        <v>-4.1338</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0.032</t>
+          <t>0.036</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>4.39</v>
+        <v>3.38</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Microservices</t>
+          <t>Monolithic</t>
         </is>
       </c>
     </row>

</xml_diff>